<commit_message>
Docs: operating schedule + Asia guide, testing report, merge summary, tracker
Tracker: OPS-01..11, ASIA-01..07, MOB-01..02, QA-01 added; UXR-10 and
UXR-11 updated. Full suite 1,843: 1,793 pass, 47 skip, 3 fail only in the
sandbox (port binding; 14/14 outside it). Test and Prod-profile servers
17/17 each.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ATIP_MASTER_TRACKER.xlsx
+++ b/ATIP_MASTER_TRACKER.xlsx
@@ -169,7 +169,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill/>
     </fill>
@@ -396,6 +396,11 @@
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -572,7 +577,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -610,6 +615,8 @@
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8326,7 +8333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I354"/>
+  <dimension ref="A1:I375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8350,12 +8357,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DONE: 122</t>
+          <t>DONE: 138</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IN PROGRESS: 182</t>
+          <t>IN PROGRESS: 187</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8370,10 +8377,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>total: 350</t>
-        </is>
-      </c>
-    </row>
+          <t>total: 371</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -24868,6 +24876,953 @@
       <c r="I354" s="12" t="inlineStr">
         <is>
           <t>dashboard/security.py; enterprise/authz.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>OPS-01</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Merge pending UI/UX changes (UXR-01..03)</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Uncommitted UXR delta reviewed and merged into master; halt-route date.today() replaced with an IST clock; 4 other dashboard branches reviewed and NOT merged (hosting/stale)</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>Owner decision on central-auth owner gate + /ATIP base path (hosting)</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>dashboard/command_page.py; dashboard/command_routes.py; orders/sessions.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>OPS-02</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Operating schedule STOPPED 21:00-06:00 IST</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py gates the schedule loop + run_job; orders.risk.halted() closes every order path; feed window + order monitor check is_stopped()</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>Watch the first real 21:00 stop on the Mac (atip.log + /api/status)</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; pipeline/scheduler.py; orders/risk.py; data/dhan_ws.py; dashboard/server.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>OPS-03</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Read-only dashboard + STOPPED banner</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Banner on /, /command, /m, /global-asia (polls /api/status 60s); writes -&gt; HTTP 423 except override, halt, sign-in</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>dashboard/global_asia.py; pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>OPS-04</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>scheduler_status table + /api/status</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>scheduler_status, scheduler_override, resume_runs, deferred_jobs; GET /api/status</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; dashboard/global_asia.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>OPS-05</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>06:00 resume sequence (6 steps, logged)</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Steps logged as resume_1..6 in pipeline_log + resume_runs.steps_json; real end-to-end run on the Prod-profile snapshot</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>Confirm on the Mac at a real 06:00 with Dhan + Anthropic keys present</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; pipeline/premarket_report.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>OPS-06</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Missed-resume catch-up + run lock</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>tick() at start-up, every 15 s and on wake; resume_runs per IST date + job_lock; crashed run re-run after 2 h</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; pipeline/scheduler.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>OPS-07</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Weekends / NSE holidays</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Step 6 SKIPPED on non-trading days; status live_feeds false</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>OPS-08</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Manual start/stop override (logged)</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>POST /api/status/override stop|start|auto (token, owner-only); CLI too; scheduler_status + alert_log</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>Add buttons on /command (API + banner done)</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>dashboard/global_asia.py; enterprise/authz.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>OPS-09</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Loud alert on keyword-classifier fallback</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Resume step 3 DEGRADED + critical alert 'NEWS SENTIMENT FALLBACK'</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>OPS-10</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Null-EMA gap for small/mid-caps</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>data/ema_gap.py fills missing sessions from the NSE Bhavcopy archive (insert-only), recomputes indicators; resume step 4</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>Reaches SMA-200 after ~1 week of 06:00 runs; verify on live DB</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>data/ema_gap.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>OPS-11</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Scheduler mechanism decision documented</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Kept ONE mechanism (in-process schedule loop) — deviation from the two named options, reasons in scheduler.py header + docs</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>Owner to confirm the decision</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>pipeline/scheduler.py; docs/OPERATING_SCHEDULE_AND_ASIA_2026-10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>ASIA-01</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Asia markets data module (6 indices, primary + fallback)</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; 14 sources probed: 11 OK, 3 FLAGGED (TOPIX Yahoo, KSE-100 PSX DPS HTTP 462, KSE-100 Yahoo); Stooq rejected (JS wall) | BLOCKER: TOPIX / KSE-100 fallback sources fail from India</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>TOPIX and KSE-100 have one working source from this network</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; data/asia_exchanges.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>ASIA-02</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>global_indices_daily + 600-day retention</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>global_indices_daily, asia_signals, asia_sentiment in LONG (600 d) purge; data-inventory classified</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; db/purge.py; enterprise/privacy.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>ASIA-03</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Exchange hours + holidays from config; 3 Asia runs</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>data/asia_exchanges.json (JPX/KRX/TWSE/PSX) + config override; runs 06:00, 10:45, 17:15 IST; calendar self-check</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>2026 holiday lists unverified (lunar dates for PSX); confirm against exchange notices</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>data/asia_exchanges.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>ASIA-04</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Per-market BULLISH/NEUTRAL/BEARISH + confidence</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>compute_signal; defect fixed in testing: no dead band made sideways tapes BULLISH</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>Back-test the thresholds on 1y of history</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>ASIA-05</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Asia Sentiment Score -&gt; Market Health + pre-market report</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>weights in asia_exchanges.json; MH weight_config ('MH','Asia') 0.05; pre-market report + 08:30 brief line</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>Owner to confirm the 0.05 MH weight</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; scores/engine.py; pipeline/premarket_report.py; alerts/telegram.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>ASIA-06</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Pakistan geopolitical / risk-event flag</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>pakistan_risk(): NONE/ELEVATED/HIGH from classified news + Google News Pakistan feed; PK_GEO_RISK weight 0.10</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; data/news.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>ASIA-07</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Global &amp; Asia tab</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Tab on /, page /global-asia, screen on /m; informational only</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>dashboard/global_asia.py; dashboard/server.py; dashboard/w38_page.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>MOB-01</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Android app: merged UI, status banner, Global &amp; Asia</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>New Kotlin shell (mobile/android): tabs Today/Command/Global &amp; Asia + native /api/status banner | BLOCKER: No Android SDK / JDK installed</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>Build + install: no Android SDK/Java on the Mac; needs Android Studio</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>mobile/android</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>MOB-02</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>iOS app: merged UI, status banner, Global &amp; Asia</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>New SwiftUI shell (mobile/ios, XcodeGen spec): same tabs + native banner; swiftc -parse OK | BLOCKER: Xcode not installed</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>Build: needs Xcode (only Command Line Tools installed); App Store needs a developer account</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>mobile/ios</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>QA-01</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Test + Prod server testing + report</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Run on local Test (ATIP_ENV=test, seeded DB, :8765) and Prod-profile (ATIP_ENV=production, live-DB snapshot, :8766) instances; full suite | BLOCKER: No hosted Test/Prod servers exist</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>Repeat on real hosted servers once they exist (GAP-2610-16)</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>docs/TEST_REPORT_2026-10-26_OPS_ASIA.md</t>
         </is>
       </c>
     </row>
@@ -26595,7 +27550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V270"/>
+  <dimension ref="A1:V291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="29.44140625" customWidth="1" min="3" max="3"/>
@@ -46944,7 +47899,6 @@
           <t>orders/rules.py; orders/sessions.py</t>
         </is>
       </c>
-      <c r="P263" t="inlineStr"/>
       <c r="Q263" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47027,7 +47981,6 @@
           <t>docs/UX_REDESIGN_2026-10.md</t>
         </is>
       </c>
-      <c r="P264" t="inlineStr"/>
       <c r="Q264" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47108,8 +48061,6 @@
           <t>Build after owner review of prototype</t>
         </is>
       </c>
-      <c r="O265" t="inlineStr"/>
-      <c r="P265" t="inlineStr"/>
       <c r="Q265" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47187,8 +48138,6 @@
           <t>Wrap orders.risk.pretrade_check dry run in a preview endpoint</t>
         </is>
       </c>
-      <c r="O266" t="inlineStr"/>
-      <c r="P266" t="inlineStr"/>
       <c r="Q266" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47261,9 +48210,6 @@
           <t>Prototype only; /trading has parts</t>
         </is>
       </c>
-      <c r="N267" t="inlineStr"/>
-      <c r="O267" t="inlineStr"/>
-      <c r="P267" t="inlineStr"/>
       <c r="Q267" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47341,8 +48287,6 @@
           <t>Needs UXR-03 rule links populated</t>
         </is>
       </c>
-      <c r="O268" t="inlineStr"/>
-      <c r="P268" t="inlineStr"/>
       <c r="Q268" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47404,15 +48348,15 @@
       </c>
       <c r="J269" s="18" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="K269" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t>No native app codebase exists; /m is a read-only PWA; /command is responsive</t>
+          <t>Native shells written (mobile/android, mobile/ios) with the status banner and Global &amp; Asia; not built — no Android SDK/Xcode on the Mac (MOB-01/02)</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
@@ -47425,7 +48369,6 @@
           <t>dashboard/w38_page.py</t>
         </is>
       </c>
-      <c r="P269" t="inlineStr"/>
       <c r="Q269" t="inlineStr">
         <is>
           <t>Claude (development)</t>
@@ -47491,11 +48434,11 @@
         </is>
       </c>
       <c r="K270" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="M270" t="inlineStr">
         <is>
-          <t>Full suite run in an isolated copy; ATIP has no Test/Prod servers yet</t>
+          <t>Tested on local Test + Prod-profile instances (QA-01); hosted servers still do not exist</t>
         </is>
       </c>
       <c r="N270" t="inlineStr">
@@ -47503,7 +48446,6 @@
           <t>Repeat on Oracle Cloud dev/test once ATIP is deployed there | BLOCKER: ATIP not yet deployed to a Test or Prod server</t>
         </is>
       </c>
-      <c r="O270" t="inlineStr"/>
       <c r="P270" t="inlineStr">
         <is>
           <t>docs/UX_TEST_REPORT_2026-10-26.md</t>
@@ -47521,6 +48463,1836 @@
         <v>46321</v>
       </c>
       <c r="V270" t="inlineStr">
+        <is>
+          <t>Testing: IN PROGRESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="n">
+        <v>13</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>OPS-01</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Merge pending UI/UX changes (UXR-01..03)</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Review + merge Command Center, kill-switch UI/API, sessions registry; no regressions</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J271" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K271" t="n">
+        <v>100</v>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>Uncommitted UXR delta reviewed and merged into master; halt-route date.today() replaced with an IST clock; 4 other dashboard branches reviewed and NOT merged (hosting/stale)</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>Owner decision on central-auth owner gate + /ATIP base path (hosting)</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>dashboard/command_page.py; dashboard/command_routes.py; orders/sessions.py</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>tests/test_ux_merge_regression.py (23); test_ux_command_center.py; HTTP smoke 17/17 Test + Prod</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S271" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T271" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U271" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V271" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="n">
+        <v>13</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>OPS-02</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Operating schedule STOPPED 21:00-06:00 IST</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>All jobs, feeds, polling, trigger monitoring paused; no order placed or triggered</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J272" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K272" t="n">
+        <v>100</v>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py gates the schedule loop + run_job; orders.risk.halted() closes every order path; feed window + order monitor check is_stopped()</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>Watch the first real 21:00 stop on the Mac (atip.log + /api/status)</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; pipeline/scheduler.py; orders/risk.py; data/dhan_ws.py; dashboard/server.py</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py (39)</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S272" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T272" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U272" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V272" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="n">
+        <v>13</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>OPS-03</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Read-only dashboard + STOPPED banner</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Banner 'ATIP stopped — resumes 06:00 IST' + last-updated; writes refused</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J273" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K273" t="n">
+        <v>100</v>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Banner on /, /command, /m, /global-asia (polls /api/status 60s); writes -&gt; HTTP 423 except override, halt, sign-in</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>dashboard/global_asia.py; pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py; HTTP smoke Test + Prod; browser 375px + desktop</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S273" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T273" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U273" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V273" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="n">
+        <v>13</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>OPS-04</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>scheduler_status table + /api/status</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Status STOPPED/RUNNING/RESUMING and every transition recorded and served</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J274" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K274" t="n">
+        <v>100</v>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>scheduler_status, scheduler_override, resume_runs, deferred_jobs; GET /api/status</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; dashboard/global_asia.py</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S274" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T274" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U274" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V274" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="n">
+        <v>13</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>OPS-05</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>06:00 resume sequence (6 steps, logged)</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Backfill -&gt; collect -&gt; sentiment -&gt; indexes -&gt; report before 08:30 -&gt; live feeds</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J275" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K275" t="n">
+        <v>95</v>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>Steps logged as resume_1..6 in pipeline_log + resume_runs.steps_json; real end-to-end run on the Prod-profile snapshot</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>Confirm on the Mac at a real 06:00 with Dhan + Anthropic keys present</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; pipeline/premarket_report.py</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py; real run log (testing report)</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S275" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T275" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U275" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V275" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="n">
+        <v>13</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>OPS-06</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Missed-resume catch-up + run lock</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Machine off at 06:00 -&gt; resume on startup/wake, never twice</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J276" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K276" t="n">
+        <v>100</v>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>tick() at start-up, every 15 s and on wake; resume_runs per IST date + job_lock; crashed run re-run after 2 h</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py; pipeline/scheduler.py</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py (catch-up, lock, duplicate, crash)</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S276" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T276" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U276" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="n">
+        <v>13</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>OPS-07</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Weekends / NSE holidays</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>06:00 collection + analysis still run; no intraday live feeds</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J277" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K277" t="n">
+        <v>100</v>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>Step 6 SKIPPED on non-trading days; status live_feeds false</t>
+        </is>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py (weekend, holiday)</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S277" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T277" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U277" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="n">
+        <v>13</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>OPS-08</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Manual start/stop override (logged)</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Override from the dashboard, logged</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J278" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K278" t="n">
+        <v>100</v>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>POST /api/status/override stop|start|auto (token, owner-only); CLI too; scheduler_status + alert_log</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>Add buttons on /command (API + banner done)</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>dashboard/global_asia.py; enterprise/authz.py</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S278" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T278" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U278" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="n">
+        <v>13</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>OPS-09</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Loud alert on keyword-classifier fallback</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Claude sentiment; fallback alerts loudly</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J279" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K279" t="n">
+        <v>100</v>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>Resume step 3 DEGRADED + critical alert 'NEWS SENTIMENT FALLBACK'</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>tests/test_operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S279" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T279" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U279" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V279" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="n">
+        <v>13</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>OPS-10</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Null-EMA gap for small/mid-caps</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>EMA-50/SMA-200 null for short-history symbols</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J280" s="17" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="K280" t="n">
+        <v>85</v>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>data/ema_gap.py fills missing sessions from the NSE Bhavcopy archive (insert-only), recomputes indicators; resume step 4</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>Reaches SMA-200 after ~1 week of 06:00 runs; verify on live DB</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>data/ema_gap.py</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>tests/test_ema_gap.py (3); real run on snapshot (testing report)</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S280" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U280" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V280" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="n">
+        <v>13</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>OPS-11</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Scheduler mechanism decision documented</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>APScheduler or Windows Task Scheduler — pick one, document why</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J281" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K281" t="n">
+        <v>100</v>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>Kept ONE mechanism (in-process schedule loop) — deviation from the two named options, reasons in scheduler.py header + docs</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>Owner to confirm the decision</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>pipeline/scheduler.py; docs/OPERATING_SCHEDULE_AND_ASIA_2026-10.md</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S281" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T281" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U281" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V281" t="inlineStr">
+        <is>
+          <t>Testing: N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="n">
+        <v>13</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>ASIA-01</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Asia markets data module (6 indices, primary + fallback)</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>KOSPI, KOSDAQ, TAIEX, Nikkei 225, TOPIX, KSE-100; verify every source</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J282" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K282" t="n">
+        <v>95</v>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; 14 sources probed: 11 OK, 3 FLAGGED (TOPIX Yahoo, KSE-100 PSX DPS HTTP 462, KSE-100 Yahoo); Stooq rejected (JS wall)</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>TOPIX and KSE-100 have one working source from this network | BLOCKER: TOPIX / KSE-100 fallback sources fail from India</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; data/asia_exchanges.json</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py (46); live verify + run</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S282" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T282" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U282" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V282" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="n">
+        <v>13</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>ASIA-02</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>global_indices_daily + 600-day retention</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Daily OHLC + session status, retention policy</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J283" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K283" t="n">
+        <v>100</v>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>global_indices_daily, asia_signals, asia_sentiment in LONG (600 d) purge; data-inventory classified</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; db/purge.py; enterprise/privacy.py</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S283" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T283" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U283" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V283" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="n">
+        <v>13</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>ASIA-03</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Exchange hours + holidays from config; 3 Asia runs</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>No hardcoded hours; 06:00 + mid-morning + post-close</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J284" s="17" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="K284" t="n">
+        <v>85</v>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>data/asia_exchanges.json (JPX/KRX/TWSE/PSX) + config override; runs 06:00, 10:45, 17:15 IST; calendar self-check</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>2026 holiday lists unverified (lunar dates for PSX); confirm against exchange notices</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>data/asia_exchanges.json</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S284" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U284" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V284" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="n">
+        <v>13</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>ASIA-04</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Per-market BULLISH/NEUTRAL/BEARISH + confidence</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Trend, momentum, volatility, gap</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J285" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K285" t="n">
+        <v>100</v>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>compute_signal; defect fixed in testing: no dead band made sideways tapes BULLISH</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>Back-test the thresholds on 1y of history</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S285" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T285" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U285" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V285" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="n">
+        <v>13</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>ASIA-05</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Asia Sentiment Score -&gt; Market Health + pre-market report</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Configurable weights</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J286" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K286" t="n">
+        <v>100</v>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>weights in asia_exchanges.json; MH weight_config ('MH','Asia') 0.05; pre-market report + 08:30 brief line</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>Owner to confirm the 0.05 MH weight</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; scores/engine.py; pipeline/premarket_report.py; alerts/telegram.py</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S286" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T286" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U286" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V286" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="n">
+        <v>13</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>ASIA-06</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Pakistan geopolitical / risk-event flag</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Separate factor driven by news sentiment</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J287" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K287" t="n">
+        <v>100</v>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>pakistan_risk(): NONE/ELEVATED/HIGH from classified news + Google News Pakistan feed; PK_GEO_RISK weight 0.10</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>data/asia_markets.py; data/news.py</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py (5 cases)</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S287" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T287" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U287" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V287" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="n">
+        <v>13</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>ASIA-07</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Global &amp; Asia tab</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Last value, % change, signal, session status</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J288" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K288" t="n">
+        <v>100</v>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Tab on /, page /global-asia, screen on /m; informational only</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>dashboard/global_asia.py; dashboard/server.py; dashboard/w38_page.py</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>tests/test_asia_markets.py; browser desktop + 375px</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S288" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="T288" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U288" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>Testing: COMPLETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="n">
+        <v>13</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>MOB-01</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Android app: merged UI, status banner, Global &amp; Asia</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Update Android app</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J289" s="22" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>60</v>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>New Kotlin shell (mobile/android): tabs Today/Command/Global &amp; Asia + native /api/status banner</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>Build + install: no Android SDK/Java on the Mac; needs Android Studio | BLOCKER: No Android SDK / JDK installed</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>mobile/android</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>not built (no toolchain)</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S289" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U289" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V289" t="inlineStr">
+        <is>
+          <t>Testing: IN PROGRESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="n">
+        <v>13</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>MOB-02</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>iOS app: merged UI, status banner, Global &amp; Asia</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Update iOS app</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J290" s="22" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K290" t="n">
+        <v>60</v>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>New SwiftUI shell (mobile/ios, XcodeGen spec): same tabs + native banner; swiftc -parse OK</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>Build: needs Xcode (only Command Line Tools installed); App Store needs a developer account | BLOCKER: Xcode not installed</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>mobile/ios</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>swiftc -parse only</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S290" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U290" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V290" t="inlineStr">
+        <is>
+          <t>Testing: IN PROGRESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="n">
+        <v>13</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Ops schedule + Asia signals (2026-10-26)</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>QA-01</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Test + Prod server testing + report</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Suite + UAT on Test and Prod</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Owner prompt 2026-10-26: UI/UX merge, operating schedule, Asia signals</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J291" s="22" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K291" t="n">
+        <v>80</v>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Run on local Test (ATIP_ENV=test, seeded DB, :8765) and Prod-profile (ATIP_ENV=production, live-DB snapshot, :8766) instances; full suite</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>Repeat on real hosted servers once they exist (GAP-2610-16) | BLOCKER: No hosted Test/Prod servers exist</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>docs/TEST_REPORT_2026-10-26_OPS_ASIA.md</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>full suite + HTTP smoke + browser</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S291" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="U291" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="V291" t="inlineStr">
         <is>
           <t>Testing: IN PROGRESS</t>
         </is>

</xml_diff>

<commit_message>
News impact estimate: Indian + world news to a session call, tracked against the close
data/news_impact.py fetches the Indian and world feeds, assesses each market-relevant
headline (Claude Haiku under the news cost cap, keyword rules as a fallback), combines
them into a 0-100 session score with sector scores, drivers and a brief, and scores
each call against the Nifty 50 and sector closes next to two naive baselines.

Shown on the News and Global & Asia tabs, /global-asia, /m, the pre-market report and
the Telegram brief. Scheduled at 07:40, 12:20, 15:50, 20:15 and on 06:00 resume,
evaluated at 16:20. Informational only: no score input, no orders.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ATIP_MASTER_TRACKER.xlsx
+++ b/ATIP_MASTER_TRACKER.xlsx
@@ -8333,7 +8333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I375"/>
+  <dimension ref="A1:I380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8357,12 +8357,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DONE: 138</t>
+          <t>DONE: 142</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IN PROGRESS: 187</t>
+          <t>IN PROGRESS: 188</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8377,11 +8377,10 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>total: 371</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>total: 376</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -25823,6 +25822,241 @@
       <c r="I375" t="inlineStr">
         <is>
           <t>docs/TEST_REPORT_2026-10-26_OPS_ASIA.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>NI-01</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Data Platform</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>News impact module: fetch + analyse</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>data/news_impact.run(): RSS_FEEDS + GLOBAL_FEEDS through run_news_pipeline (dedup, classify, store), then assess, combine, track</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>data/news_impact.py; data/news.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>NI-02</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Per-headline impact assessment</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Claude (news model + daily cap, purpose news_impact) with JSON schema; keyword-rule fallback reads crude/yield/dollar moves for India, keeps company news off the Nifty; recaps skipped | BLOCKER: ANTHROPIC_API_KEY (owner)</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Owner adds ANTHROPIC_API_KEY; then verify a live Claude run (only stubbed so far)</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>data/news_impact.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>NI-03</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Session estimate: score, bias, sectors, drivers, brief</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>0-100 score, POSITIVE/NEUTRAL/NEGATIVE + strength, per-sector scores for 11 NSE indices, top 8 drivers, Claude brief (rules fallback); informational only</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>data/news_impact.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>NI-04</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Tracking check vs Nifty close</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>news_impact_eval vs index_levels 15:30; pre-open call per session; baselines (commonest outcome, yesterday again); per-sector and per-headline hits; scheduled 07:40/12:20/15:50/20:15 + 06:00 resume, scored 16:20</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Read the track record after 20+ sessions before relying on it</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>data/news_impact.py; pipeline/scheduler.py; pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>NI-05</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>News impact panel + API</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>/api/news-impact, /accuracy, /refresh (owner token); panel on / News + Global &amp; Asia tabs, /global-asia, /m (Android/iOS apps load it); pre-market report section; Telegram brief line</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>dashboard/news_impact_view.py; dashboard/global_asia.py; dashboard/server.py; dashboard/w38_page.py; pipeline/premarket_report.py; alerts/telegram.py</t>
         </is>
       </c>
     </row>
@@ -27550,7 +27784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V291"/>
+  <dimension ref="A1:V296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="29.44140625" customWidth="1" min="3" max="3"/>
@@ -50298,6 +50532,506 @@
         </is>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="n">
+        <v>14</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>News impact estimate (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>NI-01</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Data Platform</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>News impact module: fetch + analyse</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Module pulls Indian + world feeds itself and analyses them</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: estimate news impact on the Indian market from Indian + world news</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J292" s="22" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K292" t="n">
+        <v>100</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>NS-02, GLOBAL_FEEDS</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>data/news_impact.run(): RSS_FEEDS + GLOBAL_FEEDS through run_news_pipeline (dedup, classify, store), then assess, combine, track</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>data/news_impact.py; data/news.py</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>tests/test_news_impact.py (43); live run on live-DB copy: 115 headlines fetched (29 India, 86 world)</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S292" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="U292" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="V292" t="inlineStr">
+        <is>
+          <t>Additive; informational only</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="n">
+        <v>14</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>News impact estimate (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>NI-02</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Per-headline impact assessment</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Direction, size, horizon, channel, sectors, confidence per headline</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: estimate news impact on the Indian market from Indian + world news</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J293" s="22" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="K293" t="n">
+        <v>90</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>NI-01, NS-03</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Claude (news model + daily cap, purpose news_impact) with JSON schema; keyword-rule fallback reads crude/yield/dollar moves for India, keeps company news off the Nifty; recaps skipped</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>Owner adds ANTHROPIC_API_KEY; then verify a live Claude run (only stubbed so far) | BLOCKER: ANTHROPIC_API_KEY (owner)</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>data/news_impact.py</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>tests/test_news_impact.py (43); live run on live-DB copy: 115 headlines fetched (29 India, 86 world)</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S293" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="U293" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="V293" t="inlineStr">
+        <is>
+          <t>Additive; informational only</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="n">
+        <v>14</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>News impact estimate (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>NI-03</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Session estimate: score, bias, sectors, drivers, brief</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Combine headlines into one call for the coming NSE session</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: estimate news impact on the Indian market from Indian + world news</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J294" s="22" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K294" t="n">
+        <v>100</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>NI-02</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>0-100 score, POSITIVE/NEUTRAL/NEGATIVE + strength, per-sector scores for 11 NSE indices, top 8 drivers, Claude brief (rules fallback); informational only</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>data/news_impact.py</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>tests/test_news_impact.py (43); live run on live-DB copy: 115 headlines fetched (29 India, 86 world)</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S294" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="U294" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="V294" t="inlineStr">
+        <is>
+          <t>Additive; informational only</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="n">
+        <v>14</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>News impact estimate (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>NI-04</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>AI/News</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Tracking check vs Nifty close</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Score every call against what the market did; compare with naive baselines</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: estimate news impact on the Indian market from Indian + world news</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J295" s="22" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K295" t="n">
+        <v>100</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>NI-03</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>news_impact_eval vs index_levels 15:30; pre-open call per session; baselines (commonest outcome, yesterday again); per-sector and per-headline hits; scheduled 07:40/12:20/15:50/20:15 + 06:00 resume, scored 16:20</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>Read the track record after 20+ sessions before relying on it</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>data/news_impact.py; pipeline/scheduler.py; pipeline/operating_schedule.py</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>tests/test_news_impact.py (43); live run on live-DB copy: 115 headlines fetched (29 India, 86 world)</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S295" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="U295" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="V295" t="inlineStr">
+        <is>
+          <t>Additive; informational only</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="n">
+        <v>14</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>News impact estimate (2026-10-27)</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>NI-05</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>News impact panel + API</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Show the estimate on desktop, phone and apps; pre-market report + morning brief</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: estimate news impact on the Indian market from Indian + world news</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J296" s="22" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K296" t="n">
+        <v>100</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>NI-03</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>/api/news-impact, /accuracy, /refresh (owner token); panel on / News + Global &amp; Asia tabs, /global-asia, /m (Android/iOS apps load it); pre-market report section; Telegram brief line</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>dashboard/news_impact_view.py; dashboard/global_asia.py; dashboard/server.py; dashboard/w38_page.py; pipeline/premarket_report.py; alerts/telegram.py</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>tests/test_news_impact.py (43); live run on live-DB copy: 115 headlines fetched (29 India, 86 world)</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S296" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="U296" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="V296" t="inlineStr">
+        <is>
+          <t>Additive; informational only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V259">
     <filterColumn colId="9" hiddenButton="0" showButton="1">

</xml_diff>

<commit_message>
UX console screens (UXR-06..09) and session gate in the trigger engine (UXR-04)
- /command/signals: ranked EOD signals, factor bars, plain-language why, signal vs live gap
- /command/setup: Rs risk/reward, R:R, charges, loss budget, pre-trade checklist; saves a
  confirm-gated bracket rule linked to a session
- /command/monitor: positions on a stop-price-target bar, rules watching with session holds,
  order log with causes, stale-feed banner
- /command/journal: per-session trades, win rate, avg R, P&L; hit rate by score band;
  straight-line Dec 2027 range labelled not a forecast
- orders/sessions.py gate(): entry rules of a paused/OFF/MANUAL or over-limit session are held;
  exit legs never held; unlinked rules unchanged; AUTO still does not skip the confirmation tap

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ATIP_MASTER_TRACKER.xlsx
+++ b/ATIP_MASTER_TRACKER.xlsx
@@ -8333,7 +8333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I380"/>
+  <dimension ref="A1:I385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8362,7 +8362,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IN PROGRESS: 187</t>
+          <t>IN PROGRESS: 192</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8377,11 +8377,10 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>total: 376</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>total: 381</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -26058,6 +26057,241 @@
       <c r="I380" t="inlineStr">
         <is>
           <t>dashboard/news_impact_view.py; dashboard/global_asia.py; dashboard/server.py; dashboard/w38_page.py; pipeline/premarket_report.py; alerts/telegram.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>UXR-04</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Trigger engine honours sessions</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Entry rules of a PAUSED/OFF/MANUAL or over-limit session are held (max trades, realised loss, capital cap); exit legs never held; AUTO does not skip the confirmation tap</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>Owner UAT; owner decision on AUTO bypass</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>orders/sessions.py; orders/rules.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>UXR-06</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Signal Explorer with explainability</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>/command/signals: ranked EOD signals, factor bars, plain-language why, signal vs live gap; tests/test_ux_console.py</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>Owner UAT with live data</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>dashboard/command_more.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>UXR-07</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Trade Setup with Rs risk preview</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>/command/setup: steppers, Rs risk/reward, R:R, charges, loss budget, pre-trade checklist; saves a confirm-gated bracket rule linked to a session</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>Owner UAT with live data</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>dashboard/command_more.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>UXR-08</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Live Monitor</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>/command/monitor: positions on a stop-price-target bar, rules watching with distance and session hold reason, order log with causes, stale-feed banner</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>Owner UAT with live data</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>dashboard/command_more.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>UXR-09</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Journal per session + 2027 range</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>/command/journal: per-session trades, successful, win rate, avg R, P&amp;L; hit rate by score band; straight-line Dec 2027 range labelled not a forecast</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>Owner UAT; range needs 10+ recorded sessions</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>dashboard/command_more.py; orders/sessions.py</t>
         </is>
       </c>
     </row>

</xml_diff>